<commit_message>
CMGJ-31 #time 1h Comprobacion pinout camara, timbrado con multimetro y creacion de imagen para memoria
</commit_message>
<xml_diff>
--- a/report/gfx/tables/mt9v111_pinout.xlsx
+++ b/report/gfx/tables/mt9v111_pinout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos\Documents\MSEI\TFM\report\gfx\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B12B053C-7A00-445C-A1FA-878CAFA15E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85E55328-4DFE-41C9-BFC8-0633C9C7A599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7EBFD44C-1CBA-4821-AE26-A6556F26BE7A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="58">
   <si>
     <t>T14</t>
   </si>
@@ -159,6 +159,57 @@
   </si>
   <si>
     <t>FPGA PIN2</t>
+  </si>
+  <si>
+    <t>JA</t>
+  </si>
+  <si>
+    <t>JXADC</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>L3</t>
+  </si>
+  <si>
+    <t>G2</t>
+  </si>
+  <si>
+    <t>H1</t>
+  </si>
+  <si>
+    <t>K2</t>
+  </si>
+  <si>
+    <t>G3</t>
+  </si>
+  <si>
+    <t>M2</t>
+  </si>
+  <si>
+    <t>N2</t>
+  </si>
+  <si>
+    <t>K3</t>
+  </si>
+  <si>
+    <t>M3</t>
+  </si>
+  <si>
+    <t>M1</t>
+  </si>
+  <si>
+    <t>N1</t>
   </si>
 </sst>
 </file>
@@ -174,15 +225,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -190,13 +247,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -613,8 +708,12 @@
       <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+      <c r="E2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -629,8 +728,12 @@
       <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
+      <c r="E3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -645,8 +748,12 @@
       <c r="D4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+      <c r="E4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -661,8 +768,12 @@
       <c r="D5" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
+      <c r="E5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -674,8 +785,9 @@
       <c r="D6" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
+      <c r="E6" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -687,7 +799,9 @@
       <c r="D7" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="1"/>
+      <c r="E7" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -699,8 +813,12 @@
       <c r="C8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
+      <c r="E8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -715,8 +833,12 @@
       <c r="D9" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
+      <c r="E9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -731,8 +853,12 @@
       <c r="D10" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
+      <c r="E10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -747,8 +873,12 @@
       <c r="D11" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
+      <c r="E11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -760,7 +890,9 @@
       <c r="D12" t="s">
         <v>34</v>
       </c>
-      <c r="E12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -772,7 +904,9 @@
       <c r="D13" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="1"/>
+      <c r="E13" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -787,8 +921,12 @@
       <c r="D14" t="s">
         <v>1</v>
       </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
+      <c r="E14" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -803,8 +941,12 @@
       <c r="D15" t="s">
         <v>5</v>
       </c>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
+      <c r="E15" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -819,8 +961,12 @@
       <c r="D16" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="E16" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
@@ -835,8 +981,12 @@
       <c r="D17" t="s">
         <v>13</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+      <c r="E17" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
@@ -848,7 +998,10 @@
       <c r="D18" t="s">
         <v>34</v>
       </c>
-      <c r="E18" s="1"/>
+      <c r="E18" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="4"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -860,7 +1013,10 @@
       <c r="D19" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="1"/>
+      <c r="E19" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" s="2"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -875,8 +1031,12 @@
       <c r="D20" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
+      <c r="E20" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
@@ -891,8 +1051,12 @@
       <c r="D21" t="s">
         <v>20</v>
       </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
+      <c r="E21" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
@@ -907,8 +1071,12 @@
       <c r="D22" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
+      <c r="E22" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
@@ -923,8 +1091,12 @@
       <c r="D23" t="s">
         <v>28</v>
       </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
+      <c r="E23" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
@@ -936,7 +1108,10 @@
       <c r="D24" t="s">
         <v>34</v>
       </c>
-      <c r="E24" s="1"/>
+      <c r="E24" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F24" s="3"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
@@ -948,7 +1123,10 @@
       <c r="D25" t="s">
         <v>35</v>
       </c>
-      <c r="E25" s="1"/>
+      <c r="E25" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F25" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>